<commit_message>
refactor: convert tests to vitest
</commit_message>
<xml_diff>
--- a/test/e2e-generate/richtexts/out.xlsx
+++ b/test/e2e-generate/richtexts/out.xlsx
@@ -83,7 +83,6 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font/>
   </fonts>
   <fills>
     <fill>
@@ -92,16 +91,8 @@
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill/>
   </fills>
   <borders>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
     <border>
       <left/>
       <right/>
@@ -115,9 +106,6 @@
   </cellStyleXfs>
   <cellXfs>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf fontId="1" fillId="2" borderId="1" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -402,7 +390,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s" s="1">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>

</xml_diff>